<commit_message>
Test case excel file
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -1,64 +1,104 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\test_automation\test-automation-playwright\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD0A1B14-3D88-4ADE-8DBC-BECEA899E757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name=" Test cases" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name=" Test cases" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+  <si>
+    <t>Test Case ID</t>
+  </si>
+  <si>
+    <t>Input length type</t>
+  </si>
+  <si>
+    <t>Input</t>
+  </si>
+  <si>
+    <t>Expected output</t>
+  </si>
+  <si>
+    <t>Actual output</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>POS_001</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>oya koheda yanne?</t>
+  </si>
+  <si>
+    <t>ඔයා කොහෙද යන්නේ?</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="8.5"/>
+      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="8.5"/>
     </font>
     <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="8"/>
     </font>
     <font>
+      <sz val="8"/>
+      <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-      <color theme="1"/>
-      <sz val="8"/>
     </font>
     <font>
+      <sz val="8"/>
+      <color theme="1"/>
       <name val="Iskoola Pota"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="8"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -105,114 +145,46 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -478,142 +450,110 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="49.95" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="49.95" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col width="10.88671875" customWidth="1" min="1" max="1"/>
-    <col width="22.109375" customWidth="1" min="3" max="3"/>
-    <col width="25.33203125" customWidth="1" min="4" max="4"/>
-    <col width="22.5546875" customWidth="1" min="5" max="5"/>
-    <col width="14.33203125" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="12.33203125" customWidth="1" min="9" max="10"/>
+    <col min="1" max="1" width="10.88671875" customWidth="1"/>
+    <col min="3" max="3" width="22.109375" customWidth="1"/>
+    <col min="4" max="4" width="25.33203125" customWidth="1"/>
+    <col min="5" max="5" width="22.5546875" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="9" max="10" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36.6" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Input length type</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Input</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Expected output</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Actual output</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="49.95" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>POS_001</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>oyata kohomada</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>ඔයාට කොහොමද</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>ඔයාට කොහොමද</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="49.95" customHeight="1">
-      <c r="A3" s="3" t="n"/>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-    </row>
-    <row r="4" ht="49.95" customHeight="1">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-    </row>
-    <row r="5" ht="49.95" customHeight="1">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
-    </row>
-    <row r="6" ht="49.95" customHeight="1">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="7" t="n"/>
-    </row>
-    <row r="7" ht="49.95" customHeight="1">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
-    </row>
-    <row r="8" ht="49.95" customHeight="1">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
-    </row>
-    <row r="9" ht="49.95" customHeight="1">
-      <c r="A9" s="4" t="n"/>
-      <c r="B9" s="4" t="n"/>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="4" t="n"/>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="4" t="n"/>
+    <row r="1" spans="1:6" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="6"/>
+      <c r="F2" s="7"/>
+    </row>
+    <row r="3" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+    </row>
+    <row r="5" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+    </row>
+    <row r="6" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2"/>
+      <c r="B6" s="7"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="7"/>
+    </row>
+    <row r="7" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+    </row>
+    <row r="9" spans="1:6" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>

<commit_message>
Update Assignment 1 - Test cases.xlsx
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -602,7 +602,7 @@
       <c r="E6" s="6" t="inlineStr"/>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>UI Error</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
       <c r="E10" s="6" t="inlineStr"/>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>UI Error</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
link play-wright automation scripts with test case sheet
</commit_message>
<xml_diff>
--- a/Assignment 1 - Test cases.xlsx
+++ b/Assignment 1 - Test cases.xlsx
@@ -599,7 +599,11 @@
           <t>බත් කෑවට පස්සේ සෙල්ලම් කරන්න පුලුවන්ද?</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr"/>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>බත් කෑවට පස්සේ සෙල්ලම් කරන්න පුළුවන්ද?</t>
+        </is>
+      </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
           <t>UI Error</t>
@@ -651,7 +655,11 @@
           <t>ඉක්මනට ඇඳුමක් ඇද ගන්න ගමනක් යන්න, මං එද්දි ලෑස්ති වෙලා ඉන්න.</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr"/>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>ඉක්මනට ඇඳුමක් අඬා ගන්න ගමනක් යන්න, මං එද්දි ලෑස්ති වෙලා ඉන්න.</t>
+        </is>
+      </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
           <t>UI Error</t>
@@ -703,7 +711,11 @@
           <t>රෑට කෑම ඕනේ නම් පල්ලයහට එන්න</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr"/>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>රට කෑම ඕනේ නම් පල්ලයහට එන්න</t>
+        </is>
+      </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
           <t>UI Error</t>
@@ -807,7 +819,11 @@
           <t>හොඳින් විභාගය කරන්න.</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr"/>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>හොදින් විබාගය කරන්න.</t>
+        </is>
+      </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
           <t>UI Error</t>

</xml_diff>